<commit_message>
Filter Log: drop 'Installed size if different from spec' column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/2250823/2250823_AUSTINSTONE_FilterLog.xlsx
+++ b/tracker/2250823/2250823_AUSTINSTONE_FilterLog.xlsx
@@ -45,7 +45,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -60,11 +60,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002B3C8E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,24 +153,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -185,10 +162,25 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -562,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -571,8 +563,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -587,7 +578,6 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -601,19 +591,18 @@
         </is>
       </c>
       <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Airco PM</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
+      <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -627,17 +616,16 @@
         </is>
       </c>
       <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Airco APM</t>
         </is>
       </c>
-      <c r="F3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="8" t="n"/>
       <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Phase</t>
@@ -649,15 +637,14 @@
         </is>
       </c>
       <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="F4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="8" t="n"/>
       <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -667,7 +654,6 @@
       </c>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
     </row>
     <row r="6" ht="8" customHeight="1"/>
     <row r="7" ht="34" customHeight="1">
@@ -703,11 +689,6 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Installed size if different from spec</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -740,37 +721,35 @@
         <v>8</v>
       </c>
       <c r="G8" s="12" t="n"/>
-      <c r="H8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>RTU-1A</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="7" t="n"/>
+      <c r="F9" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -800,37 +779,35 @@
         <v>8</v>
       </c>
       <c r="G10" s="12" t="n"/>
-      <c r="H10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>RTU-2A</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F11" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="F11" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -860,37 +837,35 @@
         <v>8</v>
       </c>
       <c r="G12" s="12" t="n"/>
-      <c r="H12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>RTU-1C</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F13" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="7" t="n"/>
+      <c r="F13" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -920,37 +895,35 @@
         <v>8</v>
       </c>
       <c r="G14" s="12" t="n"/>
-      <c r="H14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>RTU-2C</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F15" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G15" s="12" t="n"/>
-      <c r="H15" s="7" t="n"/>
+      <c r="F15" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -979,86 +952,82 @@
       <c r="F16" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="G16" s="11" t="n"/>
-      <c r="H16" s="13" t="n"/>
+      <c r="G16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>RTU-1B</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F17" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="7" t="n"/>
+      <c r="F17" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>RTU-2B-1</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>20x25x4</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="C18" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="n"/>
       <c r="G18" s="17" t="n"/>
-      <c r="H18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>RTU-2B-1</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
       <c r="G19" s="17" t="n"/>
-      <c r="H19" s="18" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -1087,182 +1056,174 @@
       <c r="F20" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="G20" s="11" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="G20" s="12" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>RTU-2B-2</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="C21" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="7" t="n"/>
+      <c r="F21" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>AHU-1</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>20x24x4</t>
         </is>
       </c>
-      <c r="C22" s="17" t="n">
+      <c r="C22" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="17" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
       <c r="G22" s="17" t="n"/>
-      <c r="H22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>AHU-1</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C23" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="n"/>
       <c r="G23" s="17" t="n"/>
-      <c r="H23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>20x24x4</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C24" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="17" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="16" t="n"/>
       <c r="G24" s="17" t="n"/>
-      <c r="H24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>16x20x4</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C25" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="17" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="n"/>
       <c r="G25" s="17" t="n"/>
-      <c r="H25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>20x24x2</t>
         </is>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C26" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E26" s="17" t="n"/>
-      <c r="F26" s="17" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="n"/>
       <c r="G26" s="17" t="n"/>
-      <c r="H26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>16x24x2</t>
         </is>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C27" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="17" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="n"/>
       <c r="G27" s="17" t="n"/>
-      <c r="H27" s="18" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -1271,18 +1232,16 @@
       <c r="D28" s="11" t="n"/>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="13" t="n"/>
+      <c r="G28" s="12" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="n"/>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="7" t="n"/>
+      <c r="A29" s="13" t="n"/>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -1291,18 +1250,16 @@
       <c r="D30" s="11" t="n"/>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
-      <c r="G30" s="11" t="n"/>
-      <c r="H30" s="13" t="n"/>
+      <c r="G30" s="12" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="n"/>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="7" t="n"/>
+      <c r="A31" s="13" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -1311,18 +1268,16 @@
       <c r="D32" s="11" t="n"/>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
-      <c r="G32" s="11" t="n"/>
-      <c r="H32" s="13" t="n"/>
+      <c r="G32" s="12" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="n"/>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15" t="n"/>
-      <c r="G33" s="15" t="n"/>
-      <c r="H33" s="7" t="n"/>
+      <c r="A33" s="13" t="n"/>
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n"/>
+      <c r="G33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -1331,18 +1286,16 @@
       <c r="D34" s="11" t="n"/>
       <c r="E34" s="11" t="n"/>
       <c r="F34" s="11" t="n"/>
-      <c r="G34" s="11" t="n"/>
-      <c r="H34" s="13" t="n"/>
+      <c r="G34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="n"/>
-      <c r="B35" s="15" t="n"/>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="15" t="n"/>
-      <c r="G35" s="15" t="n"/>
-      <c r="H35" s="7" t="n"/>
+      <c r="A35" s="13" t="n"/>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+      <c r="G35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -1351,18 +1304,16 @@
       <c r="D36" s="11" t="n"/>
       <c r="E36" s="11" t="n"/>
       <c r="F36" s="11" t="n"/>
-      <c r="G36" s="11" t="n"/>
-      <c r="H36" s="13" t="n"/>
+      <c r="G36" s="12" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="15" t="n"/>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15" t="n"/>
-      <c r="G37" s="15" t="n"/>
-      <c r="H37" s="7" t="n"/>
+      <c r="A37" s="13" t="n"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+      <c r="G37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -1371,18 +1322,16 @@
       <c r="D38" s="11" t="n"/>
       <c r="E38" s="11" t="n"/>
       <c r="F38" s="11" t="n"/>
-      <c r="G38" s="11" t="n"/>
-      <c r="H38" s="13" t="n"/>
+      <c r="G38" s="12" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="n"/>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="15" t="n"/>
-      <c r="G39" s="15" t="n"/>
-      <c r="H39" s="7" t="n"/>
+      <c r="A39" s="13" t="n"/>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+      <c r="G39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -1391,18 +1340,16 @@
       <c r="D40" s="11" t="n"/>
       <c r="E40" s="11" t="n"/>
       <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-      <c r="H40" s="13" t="n"/>
+      <c r="G40" s="12" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15" t="n"/>
-      <c r="G41" s="15" t="n"/>
-      <c r="H41" s="7" t="n"/>
+      <c r="A41" s="13" t="n"/>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+      <c r="G41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -1411,18 +1358,16 @@
       <c r="D42" s="11" t="n"/>
       <c r="E42" s="11" t="n"/>
       <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="13" t="n"/>
+      <c r="G42" s="12" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="n"/>
-      <c r="B43" s="15" t="n"/>
-      <c r="C43" s="15" t="n"/>
-      <c r="D43" s="15" t="n"/>
-      <c r="E43" s="15" t="n"/>
-      <c r="F43" s="15" t="n"/>
-      <c r="G43" s="15" t="n"/>
-      <c r="H43" s="7" t="n"/>
+      <c r="A43" s="13" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="14" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="14" t="n"/>
+      <c r="G43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -1431,18 +1376,16 @@
       <c r="D44" s="11" t="n"/>
       <c r="E44" s="11" t="n"/>
       <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
-      <c r="H44" s="13" t="n"/>
+      <c r="G44" s="12" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="n"/>
-      <c r="B45" s="15" t="n"/>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
-      <c r="F45" s="15" t="n"/>
-      <c r="G45" s="15" t="n"/>
-      <c r="H45" s="7" t="n"/>
+      <c r="A45" s="13" t="n"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="14" t="n"/>
+      <c r="G45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -1451,29 +1394,27 @@
       <c r="D46" s="11" t="n"/>
       <c r="E46" s="11" t="n"/>
       <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
-      <c r="H46" s="13" t="n"/>
+      <c r="G46" s="12" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="n"/>
-      <c r="B47" s="15" t="n"/>
-      <c r="C47" s="15" t="n"/>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="15" t="n"/>
-      <c r="F47" s="15" t="n"/>
-      <c r="G47" s="15" t="n"/>
-      <c r="H47" s="7" t="n"/>
+      <c r="A47" s="13" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="14" t="n"/>
+      <c r="G47" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D8:D47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1557,7 +1498,7 @@
         </is>
       </c>
       <c r="I2" s="4">
-        <f>IF('Filter Log'!F2="","",'Filter Log'!F2)</f>
+        <f>IF('Filter Log'!E2="","",'Filter Log'!E2)</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -1587,7 +1528,7 @@
         </is>
       </c>
       <c r="I3" s="7">
-        <f>IF('Filter Log'!F3="","",'Filter Log'!F3)</f>
+        <f>IF('Filter Log'!E3="","",'Filter Log'!E3)</f>
         <v/>
       </c>
       <c r="J3" s="8" t="n"/>
@@ -1617,7 +1558,7 @@
         </is>
       </c>
       <c r="I4" s="7">
-        <f>IF('Filter Log'!F4="","",'Filter Log'!F4)</f>
+        <f>IF('Filter Log'!E4="","",'Filter Log'!E4)</f>
         <v/>
       </c>
       <c r="J4" s="8" t="n"/>
@@ -1716,12 +1657,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Angel Leon</t>
         </is>
@@ -1731,7 +1672,7 @@
           <t>2nd</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Tex Air Austin</t>
         </is>
@@ -1749,7 +1690,7 @@
       <c r="G8" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="19" t="n">
         <v>98.23999999999999</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -1760,26 +1701,26 @@
       <c r="J8" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K8" s="20" t="n">
+      <c r="K8" s="19" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="L8" s="20">
+      <c r="L8" s="19">
         <f>J8*K8</f>
         <v/>
       </c>
-      <c r="M8" s="13" t="inlineStr">
+      <c r="M8" s="12" t="inlineStr">
         <is>
           <t>Customer pickup</t>
         </is>
       </c>
-      <c r="N8" s="13" t="inlineStr">
+      <c r="N8" s="12" t="inlineStr">
         <is>
           <t>Urgent, units unknown at time of order.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -1789,7 +1730,7 @@
           <t>Angel Leon</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
@@ -1799,32 +1740,32 @@
           <t>Tex Air Austin</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>766028</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>380118</t>
         </is>
       </c>
-      <c r="G9" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="G9" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K9" s="22" t="n">
+      <c r="K9" s="21" t="n">
         <v>7.46</v>
       </c>
-      <c r="L9" s="22">
+      <c r="L9" s="21">
         <f>J9*K9</f>
         <v/>
       </c>
@@ -1836,12 +1777,12 @@
       <c r="N9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Angel Leon</t>
         </is>
@@ -1851,7 +1792,7 @@
           <t>2nd</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Tex Air Austin</t>
         </is>
@@ -1869,7 +1810,7 @@
       <c r="G10" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="19" t="n">
         <v>368.44</v>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -1880,26 +1821,26 @@
       <c r="J10" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="K10" s="20" t="n">
+      <c r="K10" s="19" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="L10" s="20">
+      <c r="L10" s="19">
         <f>J10*K10</f>
         <v/>
       </c>
-      <c r="M10" s="13" t="inlineStr">
+      <c r="M10" s="12" t="inlineStr">
         <is>
           <t>Delivered 2026-10-09</t>
         </is>
       </c>
-      <c r="N10" s="13" t="inlineStr">
+      <c r="N10" s="12" t="inlineStr">
         <is>
           <t>Units unknown at time of order.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
@@ -1909,7 +1850,7 @@
           <t>Angel Leon</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
@@ -1919,32 +1860,32 @@
           <t>Tex Air Austin</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>770738</t>
         </is>
       </c>
-      <c r="F11" s="15" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>382244</t>
         </is>
       </c>
-      <c r="G11" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="15" t="inlineStr">
+      <c r="G11" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H11" s="21" t="n"/>
+      <c r="I11" s="14" t="inlineStr">
         <is>
           <t>20x25x2</t>
         </is>
       </c>
-      <c r="J11" s="15" t="n">
+      <c r="J11" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="K11" s="22" t="n">
+      <c r="K11" s="21" t="n">
         <v>4.83</v>
       </c>
-      <c r="L11" s="22">
+      <c r="L11" s="21">
         <f>J11*K11</f>
         <v/>
       </c>
@@ -1956,12 +1897,12 @@
       <c r="N11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Angel Leon</t>
         </is>
@@ -1971,7 +1912,7 @@
           <t>2nd</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Tex Air Austin</t>
         </is>
@@ -1989,7 +1930,7 @@
       <c r="G12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H12" s="20" t="n"/>
+      <c r="H12" s="19" t="n"/>
       <c r="I12" s="11" t="inlineStr">
         <is>
           <t>20x20x4</t>
@@ -1998,22 +1939,22 @@
       <c r="J12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K12" s="20" t="n">
+      <c r="K12" s="19" t="n">
         <v>7.46</v>
       </c>
-      <c r="L12" s="20">
+      <c r="L12" s="19">
         <f>J12*K12</f>
         <v/>
       </c>
-      <c r="M12" s="13" t="inlineStr">
+      <c r="M12" s="12" t="inlineStr">
         <is>
           <t>Delivered 2026-10-09</t>
         </is>
       </c>
-      <c r="N12" s="13" t="n"/>
+      <c r="N12" s="12" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
@@ -2023,7 +1964,7 @@
           <t>Angel Leon</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
@@ -2033,32 +1974,32 @@
           <t>Tex Air Austin</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>770738</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>382244</t>
         </is>
       </c>
-      <c r="G13" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="15" t="inlineStr">
+      <c r="G13" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" s="21" t="n"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="J13" s="15" t="n">
+      <c r="J13" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="K13" s="22" t="n">
+      <c r="K13" s="21" t="n">
         <v>4.67</v>
       </c>
-      <c r="L13" s="22">
+      <c r="L13" s="21">
         <f>J13*K13</f>
         <v/>
       </c>
@@ -2070,37 +2011,37 @@
       <c r="N13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="13" t="n"/>
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="12" t="n"/>
       <c r="C14" s="11" t="n"/>
-      <c r="D14" s="13" t="n"/>
+      <c r="D14" s="12" t="n"/>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
       <c r="G14" s="11" t="n"/>
-      <c r="H14" s="20" t="n"/>
+      <c r="H14" s="19" t="n"/>
       <c r="I14" s="11" t="n"/>
       <c r="J14" s="11" t="n"/>
-      <c r="K14" s="20" t="n"/>
-      <c r="L14" s="20">
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19">
         <f>IF(OR(J14="",K14=""),"",J14*K14)</f>
         <v/>
       </c>
-      <c r="M14" s="13" t="n"/>
-      <c r="N14" s="13" t="n"/>
+      <c r="M14" s="12" t="n"/>
+      <c r="N14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="n"/>
+      <c r="A15" s="20" t="n"/>
       <c r="B15" s="7" t="n"/>
-      <c r="C15" s="15" t="n"/>
+      <c r="C15" s="14" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="15" t="n"/>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="22" t="n"/>
-      <c r="L15" s="22">
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n"/>
+      <c r="G15" s="14" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="14" t="n"/>
+      <c r="J15" s="14" t="n"/>
+      <c r="K15" s="21" t="n"/>
+      <c r="L15" s="21">
         <f>IF(OR(J15="",K15=""),"",J15*K15)</f>
         <v/>
       </c>
@@ -2108,37 +2049,37 @@
       <c r="N15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="13" t="n"/>
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="12" t="n"/>
       <c r="C16" s="11" t="n"/>
-      <c r="D16" s="13" t="n"/>
+      <c r="D16" s="12" t="n"/>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>
       <c r="G16" s="11" t="n"/>
-      <c r="H16" s="20" t="n"/>
+      <c r="H16" s="19" t="n"/>
       <c r="I16" s="11" t="n"/>
       <c r="J16" s="11" t="n"/>
-      <c r="K16" s="20" t="n"/>
-      <c r="L16" s="20">
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19">
         <f>IF(OR(J16="",K16=""),"",J16*K16)</f>
         <v/>
       </c>
-      <c r="M16" s="13" t="n"/>
-      <c r="N16" s="13" t="n"/>
+      <c r="M16" s="12" t="n"/>
+      <c r="N16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="n"/>
+      <c r="A17" s="20" t="n"/>
       <c r="B17" s="7" t="n"/>
-      <c r="C17" s="15" t="n"/>
+      <c r="C17" s="14" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="22" t="n"/>
-      <c r="L17" s="22">
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="14" t="n"/>
+      <c r="J17" s="14" t="n"/>
+      <c r="K17" s="21" t="n"/>
+      <c r="L17" s="21">
         <f>IF(OR(J17="",K17=""),"",J17*K17)</f>
         <v/>
       </c>
@@ -2146,37 +2087,37 @@
       <c r="N17" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="13" t="n"/>
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="12" t="n"/>
       <c r="C18" s="11" t="n"/>
-      <c r="D18" s="13" t="n"/>
+      <c r="D18" s="12" t="n"/>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
-      <c r="H18" s="20" t="n"/>
+      <c r="H18" s="19" t="n"/>
       <c r="I18" s="11" t="n"/>
       <c r="J18" s="11" t="n"/>
-      <c r="K18" s="20" t="n"/>
-      <c r="L18" s="20">
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19">
         <f>IF(OR(J18="",K18=""),"",J18*K18)</f>
         <v/>
       </c>
-      <c r="M18" s="13" t="n"/>
-      <c r="N18" s="13" t="n"/>
+      <c r="M18" s="12" t="n"/>
+      <c r="N18" s="12" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="n"/>
+      <c r="A19" s="20" t="n"/>
       <c r="B19" s="7" t="n"/>
-      <c r="C19" s="15" t="n"/>
+      <c r="C19" s="14" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="15" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="22" t="n"/>
-      <c r="L19" s="22">
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="14" t="n"/>
+      <c r="J19" s="14" t="n"/>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21">
         <f>IF(OR(J19="",K19=""),"",J19*K19)</f>
         <v/>
       </c>
@@ -2184,37 +2125,37 @@
       <c r="N19" s="7" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="13" t="n"/>
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="12" t="n"/>
       <c r="C20" s="11" t="n"/>
-      <c r="D20" s="13" t="n"/>
+      <c r="D20" s="12" t="n"/>
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
-      <c r="H20" s="20" t="n"/>
+      <c r="H20" s="19" t="n"/>
       <c r="I20" s="11" t="n"/>
       <c r="J20" s="11" t="n"/>
-      <c r="K20" s="20" t="n"/>
-      <c r="L20" s="20">
+      <c r="K20" s="19" t="n"/>
+      <c r="L20" s="19">
         <f>IF(OR(J20="",K20=""),"",J20*K20)</f>
         <v/>
       </c>
-      <c r="M20" s="13" t="n"/>
-      <c r="N20" s="13" t="n"/>
+      <c r="M20" s="12" t="n"/>
+      <c r="N20" s="12" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="n"/>
+      <c r="A21" s="20" t="n"/>
       <c r="B21" s="7" t="n"/>
-      <c r="C21" s="15" t="n"/>
+      <c r="C21" s="14" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="15" t="n"/>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="22" t="n"/>
-      <c r="I21" s="15" t="n"/>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="22" t="n"/>
-      <c r="L21" s="22">
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="21" t="n"/>
+      <c r="I21" s="14" t="n"/>
+      <c r="J21" s="14" t="n"/>
+      <c r="K21" s="21" t="n"/>
+      <c r="L21" s="21">
         <f>IF(OR(J21="",K21=""),"",J21*K21)</f>
         <v/>
       </c>
@@ -2222,37 +2163,37 @@
       <c r="N21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="13" t="n"/>
+      <c r="A22" s="18" t="n"/>
+      <c r="B22" s="12" t="n"/>
       <c r="C22" s="11" t="n"/>
-      <c r="D22" s="13" t="n"/>
+      <c r="D22" s="12" t="n"/>
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
-      <c r="H22" s="20" t="n"/>
+      <c r="H22" s="19" t="n"/>
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
-      <c r="K22" s="20" t="n"/>
-      <c r="L22" s="20">
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19">
         <f>IF(OR(J22="",K22=""),"",J22*K22)</f>
         <v/>
       </c>
-      <c r="M22" s="13" t="n"/>
-      <c r="N22" s="13" t="n"/>
+      <c r="M22" s="12" t="n"/>
+      <c r="N22" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="n"/>
+      <c r="A23" s="20" t="n"/>
       <c r="B23" s="7" t="n"/>
-      <c r="C23" s="15" t="n"/>
+      <c r="C23" s="14" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="15" t="n"/>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="15" t="n"/>
-      <c r="H23" s="22" t="n"/>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="22" t="n"/>
-      <c r="L23" s="22">
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
+      <c r="G23" s="14" t="n"/>
+      <c r="H23" s="21" t="n"/>
+      <c r="I23" s="14" t="n"/>
+      <c r="J23" s="14" t="n"/>
+      <c r="K23" s="21" t="n"/>
+      <c r="L23" s="21">
         <f>IF(OR(J23="",K23=""),"",J23*K23)</f>
         <v/>
       </c>
@@ -2260,37 +2201,37 @@
       <c r="N23" s="7" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="13" t="n"/>
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="12" t="n"/>
       <c r="C24" s="11" t="n"/>
-      <c r="D24" s="13" t="n"/>
+      <c r="D24" s="12" t="n"/>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
-      <c r="H24" s="20" t="n"/>
+      <c r="H24" s="19" t="n"/>
       <c r="I24" s="11" t="n"/>
       <c r="J24" s="11" t="n"/>
-      <c r="K24" s="20" t="n"/>
-      <c r="L24" s="20">
+      <c r="K24" s="19" t="n"/>
+      <c r="L24" s="19">
         <f>IF(OR(J24="",K24=""),"",J24*K24)</f>
         <v/>
       </c>
-      <c r="M24" s="13" t="n"/>
-      <c r="N24" s="13" t="n"/>
+      <c r="M24" s="12" t="n"/>
+      <c r="N24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="n"/>
+      <c r="A25" s="20" t="n"/>
       <c r="B25" s="7" t="n"/>
-      <c r="C25" s="15" t="n"/>
+      <c r="C25" s="14" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="15" t="n"/>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="22" t="n"/>
-      <c r="L25" s="22">
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="n"/>
+      <c r="G25" s="14" t="n"/>
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="14" t="n"/>
+      <c r="J25" s="14" t="n"/>
+      <c r="K25" s="21" t="n"/>
+      <c r="L25" s="21">
         <f>IF(OR(J25="",K25=""),"",J25*K25)</f>
         <v/>
       </c>
@@ -2298,37 +2239,37 @@
       <c r="N25" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="13" t="n"/>
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="12" t="n"/>
       <c r="C26" s="11" t="n"/>
-      <c r="D26" s="13" t="n"/>
+      <c r="D26" s="12" t="n"/>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
-      <c r="H26" s="20" t="n"/>
+      <c r="H26" s="19" t="n"/>
       <c r="I26" s="11" t="n"/>
       <c r="J26" s="11" t="n"/>
-      <c r="K26" s="20" t="n"/>
-      <c r="L26" s="20">
+      <c r="K26" s="19" t="n"/>
+      <c r="L26" s="19">
         <f>IF(OR(J26="",K26=""),"",J26*K26)</f>
         <v/>
       </c>
-      <c r="M26" s="13" t="n"/>
-      <c r="N26" s="13" t="n"/>
+      <c r="M26" s="12" t="n"/>
+      <c r="N26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="n"/>
+      <c r="A27" s="20" t="n"/>
       <c r="B27" s="7" t="n"/>
-      <c r="C27" s="15" t="n"/>
+      <c r="C27" s="14" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="15" t="n"/>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="15" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="22" t="n"/>
-      <c r="L27" s="22">
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="14" t="n"/>
+      <c r="G27" s="14" t="n"/>
+      <c r="H27" s="21" t="n"/>
+      <c r="I27" s="14" t="n"/>
+      <c r="J27" s="14" t="n"/>
+      <c r="K27" s="21" t="n"/>
+      <c r="L27" s="21">
         <f>IF(OR(J27="",K27=""),"",J27*K27)</f>
         <v/>
       </c>
@@ -2336,37 +2277,37 @@
       <c r="N27" s="7" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="13" t="n"/>
+      <c r="A28" s="18" t="n"/>
+      <c r="B28" s="12" t="n"/>
       <c r="C28" s="11" t="n"/>
-      <c r="D28" s="13" t="n"/>
+      <c r="D28" s="12" t="n"/>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
       <c r="G28" s="11" t="n"/>
-      <c r="H28" s="20" t="n"/>
+      <c r="H28" s="19" t="n"/>
       <c r="I28" s="11" t="n"/>
       <c r="J28" s="11" t="n"/>
-      <c r="K28" s="20" t="n"/>
-      <c r="L28" s="20">
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="19">
         <f>IF(OR(J28="",K28=""),"",J28*K28)</f>
         <v/>
       </c>
-      <c r="M28" s="13" t="n"/>
-      <c r="N28" s="13" t="n"/>
+      <c r="M28" s="12" t="n"/>
+      <c r="N28" s="12" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="n"/>
+      <c r="A29" s="20" t="n"/>
       <c r="B29" s="7" t="n"/>
-      <c r="C29" s="15" t="n"/>
+      <c r="C29" s="14" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="22" t="n"/>
-      <c r="I29" s="15" t="n"/>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="22" t="n"/>
-      <c r="L29" s="22">
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="21" t="n"/>
+      <c r="I29" s="14" t="n"/>
+      <c r="J29" s="14" t="n"/>
+      <c r="K29" s="21" t="n"/>
+      <c r="L29" s="21">
         <f>IF(OR(J29="",K29=""),"",J29*K29)</f>
         <v/>
       </c>
@@ -2374,37 +2315,37 @@
       <c r="N29" s="7" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="13" t="n"/>
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="12" t="n"/>
       <c r="C30" s="11" t="n"/>
-      <c r="D30" s="13" t="n"/>
+      <c r="D30" s="12" t="n"/>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
-      <c r="H30" s="20" t="n"/>
+      <c r="H30" s="19" t="n"/>
       <c r="I30" s="11" t="n"/>
       <c r="J30" s="11" t="n"/>
-      <c r="K30" s="20" t="n"/>
-      <c r="L30" s="20">
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19">
         <f>IF(OR(J30="",K30=""),"",J30*K30)</f>
         <v/>
       </c>
-      <c r="M30" s="13" t="n"/>
-      <c r="N30" s="13" t="n"/>
+      <c r="M30" s="12" t="n"/>
+      <c r="N30" s="12" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="n"/>
+      <c r="A31" s="20" t="n"/>
       <c r="B31" s="7" t="n"/>
-      <c r="C31" s="15" t="n"/>
+      <c r="C31" s="14" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="22" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="22" t="n"/>
-      <c r="L31" s="22">
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="21" t="n"/>
+      <c r="I31" s="14" t="n"/>
+      <c r="J31" s="14" t="n"/>
+      <c r="K31" s="21" t="n"/>
+      <c r="L31" s="21">
         <f>IF(OR(J31="",K31=""),"",J31*K31)</f>
         <v/>
       </c>
@@ -2412,37 +2353,37 @@
       <c r="N31" s="7" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="n"/>
-      <c r="B32" s="13" t="n"/>
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="11" t="n"/>
-      <c r="D32" s="13" t="n"/>
+      <c r="D32" s="12" t="n"/>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
       <c r="G32" s="11" t="n"/>
-      <c r="H32" s="20" t="n"/>
+      <c r="H32" s="19" t="n"/>
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="11" t="n"/>
-      <c r="K32" s="20" t="n"/>
-      <c r="L32" s="20">
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="19">
         <f>IF(OR(J32="",K32=""),"",J32*K32)</f>
         <v/>
       </c>
-      <c r="M32" s="13" t="n"/>
-      <c r="N32" s="13" t="n"/>
+      <c r="M32" s="12" t="n"/>
+      <c r="N32" s="12" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="n"/>
+      <c r="A33" s="20" t="n"/>
       <c r="B33" s="7" t="n"/>
-      <c r="C33" s="15" t="n"/>
+      <c r="C33" s="14" t="n"/>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15" t="n"/>
-      <c r="G33" s="15" t="n"/>
-      <c r="H33" s="22" t="n"/>
-      <c r="I33" s="15" t="n"/>
-      <c r="J33" s="15" t="n"/>
-      <c r="K33" s="22" t="n"/>
-      <c r="L33" s="22">
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="21" t="n"/>
+      <c r="I33" s="14" t="n"/>
+      <c r="J33" s="14" t="n"/>
+      <c r="K33" s="21" t="n"/>
+      <c r="L33" s="21">
         <f>IF(OR(J33="",K33=""),"",J33*K33)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Filter Log: PM layout (Equipment Tag, Filter Type, Date Changed) and alignment fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/2250823/2250823_AUSTINSTONE_FilterLog.xlsx
+++ b/tracker/2250823/2250823_AUSTINSTONE_FilterLog.xlsx
@@ -132,62 +132,68 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,16 +560,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -578,6 +586,8 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -591,18 +601,20 @@
         </is>
       </c>
       <c r="C2" s="5" t="n"/>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Airco PM</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -616,16 +628,18 @@
         </is>
       </c>
       <c r="C3" s="8" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Airco APM</t>
         </is>
       </c>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Phase</t>
@@ -637,14 +651,16 @@
         </is>
       </c>
       <c r="C4" s="8" t="n"/>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="8" t="n"/>
+      <c r="I4" s="8" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -654,777 +670,872 @@
       </c>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
     </row>
     <row r="6" ht="8" customHeight="1"/>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Equipment Tag</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
+          <t>Filter Type (Pre or final)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
           <t>Filter size (W x L x D)</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>MERV</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Filter set or reason</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>MERV</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Date Changed</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>RTU-1A</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>20x25x2</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="13" t="n"/>
+      <c r="I8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>RTU-1A</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>RTU-2A</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>20x25x2</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="14" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>RTU-2A</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="E11" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F11" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>RTU-1C</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>20x25x2</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>RTU-1C</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="G13" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F13" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>RTU-2C</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>20x25x2</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>RTU-2C</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="D15" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="G15" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>RTU-1B</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>20x25x4</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F16" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>RTU-1B</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="D17" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="E17" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>RTU-2B-1</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>20x25x4</t>
         </is>
       </c>
-      <c r="C18" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="18" t="n"/>
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E18" s="16" t="n"/>
-      <c r="F18" s="16" t="n"/>
-      <c r="G18" s="17" t="n"/>
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="20" t="n"/>
+      <c r="I18" s="21" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>RTU-2B-1</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C19" s="16" t="n">
+      <c r="D19" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="17" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="21" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>RTU-2B-2</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>20x25x4</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F20" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="14" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>RTU-2B-2</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="D21" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="E21" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="F21" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="17" t="n"/>
+      <c r="I21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>AHU-1</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>20x24x4</t>
         </is>
       </c>
-      <c r="C22" s="16" t="n">
+      <c r="D22" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
-      <c r="G22" s="17" t="n"/>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="20" t="n"/>
+      <c r="I22" s="21" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>AHU-1</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="C23" s="16" t="n">
+      <c r="D23" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="17" t="n"/>
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="20" t="n"/>
+      <c r="I23" s="21" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>20x24x4</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="D24" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="16" t="n"/>
-      <c r="G24" s="17" t="n"/>
+      <c r="G24" s="18" t="n"/>
+      <c r="H24" s="20" t="n"/>
+      <c r="I24" s="21" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>16x20x4</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n">
+      <c r="D25" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="17" t="n"/>
+      <c r="G25" s="18" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="21" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>20x24x2</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n">
+      <c r="D26" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="16" t="inlineStr">
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="17" t="n"/>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="21" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>ERV-1</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>16x24x2</t>
         </is>
       </c>
-      <c r="C27" s="16" t="n">
+      <c r="D27" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="16" t="inlineStr">
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
-      <c r="G27" s="17" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="21" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n"/>
-      <c r="B28" s="11" t="n"/>
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="12" t="n"/>
       <c r="C28" s="11" t="n"/>
       <c r="D28" s="11" t="n"/>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
-      <c r="G28" s="12" t="n"/>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="7" t="n"/>
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="17" t="n"/>
+      <c r="I29" s="7" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n"/>
-      <c r="B30" s="11" t="n"/>
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="12" t="n"/>
       <c r="C30" s="11" t="n"/>
       <c r="D30" s="11" t="n"/>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
-      <c r="G30" s="12" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="7" t="n"/>
+      <c r="A31" s="15" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="7" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n"/>
-      <c r="B32" s="11" t="n"/>
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="11" t="n"/>
       <c r="D32" s="11" t="n"/>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
-      <c r="G32" s="12" t="n"/>
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="14" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n"/>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="7" t="n"/>
+      <c r="A33" s="15" t="n"/>
+      <c r="B33" s="16" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="7" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="n"/>
-      <c r="B34" s="11" t="n"/>
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="12" t="n"/>
       <c r="C34" s="11" t="n"/>
       <c r="D34" s="11" t="n"/>
       <c r="E34" s="11" t="n"/>
       <c r="F34" s="11" t="n"/>
-      <c r="G34" s="12" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="14" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n"/>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="14" t="n"/>
-      <c r="G35" s="7" t="n"/>
+      <c r="A35" s="15" t="n"/>
+      <c r="B35" s="16" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="15" t="n"/>
+      <c r="H35" s="17" t="n"/>
+      <c r="I35" s="7" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="11" t="n"/>
+      <c r="A36" s="11" t="n"/>
+      <c r="B36" s="12" t="n"/>
       <c r="C36" s="11" t="n"/>
       <c r="D36" s="11" t="n"/>
       <c r="E36" s="11" t="n"/>
       <c r="F36" s="11" t="n"/>
-      <c r="G36" s="12" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="14" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n"/>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="14" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="14" t="n"/>
-      <c r="G37" s="7" t="n"/>
+      <c r="A37" s="15" t="n"/>
+      <c r="B37" s="16" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="17" t="n"/>
+      <c r="I37" s="7" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="n"/>
-      <c r="B38" s="11" t="n"/>
+      <c r="A38" s="11" t="n"/>
+      <c r="B38" s="12" t="n"/>
       <c r="C38" s="11" t="n"/>
       <c r="D38" s="11" t="n"/>
       <c r="E38" s="11" t="n"/>
       <c r="F38" s="11" t="n"/>
-      <c r="G38" s="12" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="13" t="n"/>
+      <c r="I38" s="14" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n"/>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="7" t="n"/>
+      <c r="A39" s="15" t="n"/>
+      <c r="B39" s="16" t="n"/>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="15" t="n"/>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="7" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n"/>
-      <c r="B40" s="11" t="n"/>
+      <c r="A40" s="11" t="n"/>
+      <c r="B40" s="12" t="n"/>
       <c r="C40" s="11" t="n"/>
       <c r="D40" s="11" t="n"/>
       <c r="E40" s="11" t="n"/>
       <c r="F40" s="11" t="n"/>
-      <c r="G40" s="12" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="13" t="n"/>
+      <c r="I40" s="14" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="n"/>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="14" t="n"/>
-      <c r="E41" s="14" t="n"/>
-      <c r="F41" s="14" t="n"/>
-      <c r="G41" s="7" t="n"/>
+      <c r="A41" s="15" t="n"/>
+      <c r="B41" s="16" t="n"/>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="15" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="15" t="n"/>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="7" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="n"/>
-      <c r="B42" s="11" t="n"/>
+      <c r="A42" s="11" t="n"/>
+      <c r="B42" s="12" t="n"/>
       <c r="C42" s="11" t="n"/>
       <c r="D42" s="11" t="n"/>
       <c r="E42" s="11" t="n"/>
       <c r="F42" s="11" t="n"/>
-      <c r="G42" s="12" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="13" t="n"/>
+      <c r="I42" s="14" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="n"/>
-      <c r="B43" s="14" t="n"/>
-      <c r="C43" s="14" t="n"/>
-      <c r="D43" s="14" t="n"/>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="14" t="n"/>
-      <c r="G43" s="7" t="n"/>
+      <c r="A43" s="15" t="n"/>
+      <c r="B43" s="16" t="n"/>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="15" t="n"/>
+      <c r="G43" s="15" t="n"/>
+      <c r="H43" s="17" t="n"/>
+      <c r="I43" s="7" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="n"/>
-      <c r="B44" s="11" t="n"/>
+      <c r="A44" s="11" t="n"/>
+      <c r="B44" s="12" t="n"/>
       <c r="C44" s="11" t="n"/>
       <c r="D44" s="11" t="n"/>
       <c r="E44" s="11" t="n"/>
       <c r="F44" s="11" t="n"/>
-      <c r="G44" s="12" t="n"/>
+      <c r="G44" s="11" t="n"/>
+      <c r="H44" s="13" t="n"/>
+      <c r="I44" s="14" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="n"/>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="14" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="14" t="n"/>
-      <c r="G45" s="7" t="n"/>
+      <c r="A45" s="15" t="n"/>
+      <c r="B45" s="16" t="n"/>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="15" t="n"/>
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="15" t="n"/>
+      <c r="H45" s="17" t="n"/>
+      <c r="I45" s="7" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="n"/>
-      <c r="B46" s="11" t="n"/>
+      <c r="A46" s="11" t="n"/>
+      <c r="B46" s="12" t="n"/>
       <c r="C46" s="11" t="n"/>
       <c r="D46" s="11" t="n"/>
       <c r="E46" s="11" t="n"/>
       <c r="F46" s="11" t="n"/>
-      <c r="G46" s="12" t="n"/>
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="13" t="n"/>
+      <c r="I46" s="14" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="n"/>
-      <c r="B47" s="14" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="14" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="14" t="n"/>
-      <c r="G47" s="7" t="n"/>
+      <c r="A47" s="15" t="n"/>
+      <c r="B47" s="16" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="17" t="n"/>
+      <c r="I47" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="D8:D47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="B8:B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pre,Final"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E8:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"8,13"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F8:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Needs filters,Ordered,Replaced,Not replaced,Washable - not replaced"</formula1>
     </dataValidation>
-    <dataValidation sqref="E8:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G8:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1st (media roll),2nd,3rd,Attic stock,RFI,Change order"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F8:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"8,13"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1498,7 +1609,7 @@
         </is>
       </c>
       <c r="I2" s="4">
-        <f>IF('Filter Log'!E2="","",'Filter Log'!E2)</f>
+        <f>IF('Filter Log'!G2="","",'Filter Log'!G2)</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -1528,7 +1639,7 @@
         </is>
       </c>
       <c r="I3" s="7">
-        <f>IF('Filter Log'!E3="","",'Filter Log'!E3)</f>
+        <f>IF('Filter Log'!G3="","",'Filter Log'!G3)</f>
         <v/>
       </c>
       <c r="J3" s="8" t="n"/>
@@ -1558,7 +1669,7 @@
         </is>
       </c>
       <c r="I4" s="7">
-        <f>IF('Filter Log'!E4="","",'Filter Log'!E4)</f>
+        <f>IF('Filter Log'!G4="","",'Filter Log'!G4)</f>
         <v/>
       </c>
       <c r="J4" s="8" t="n"/>
@@ -1650,14 +1761,14 @@
           <t>Delivery</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="N7" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -1690,7 +1801,7 @@
       <c r="G8" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="22" t="n">
         <v>98.23999999999999</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -1701,10 +1812,10 @@
       <c r="J8" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="22" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="L8" s="19">
+      <c r="L8" s="22">
         <f>J8*K8</f>
         <v/>
       </c>
@@ -1713,63 +1824,63 @@
           <t>Customer pickup</t>
         </is>
       </c>
-      <c r="N8" s="12" t="inlineStr">
+      <c r="N8" s="14" t="inlineStr">
         <is>
           <t>Urgent, units unknown at time of order.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Angel Leon</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Tex Air Austin</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>766028</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>380118</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="21" t="n"/>
-      <c r="I9" s="14" t="inlineStr">
+      <c r="G9" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="23" t="n"/>
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>20x20x4</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K9" s="21" t="n">
+      <c r="K9" s="23" t="n">
         <v>7.46</v>
       </c>
-      <c r="L9" s="21">
+      <c r="L9" s="23">
         <f>J9*K9</f>
         <v/>
       </c>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="M9" s="16" t="inlineStr">
         <is>
           <t>Customer pickup</t>
         </is>
@@ -1777,7 +1888,7 @@
       <c r="N9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
@@ -1810,7 +1921,7 @@
       <c r="G10" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="22" t="n">
         <v>368.44</v>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -1821,10 +1932,10 @@
       <c r="J10" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="22" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="L10" s="19">
+      <c r="L10" s="22">
         <f>J10*K10</f>
         <v/>
       </c>
@@ -1833,63 +1944,63 @@
           <t>Delivered 2026-10-09</t>
         </is>
       </c>
-      <c r="N10" s="12" t="inlineStr">
+      <c r="N10" s="14" t="inlineStr">
         <is>
           <t>Units unknown at time of order.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Angel Leon</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Tex Air Austin</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>770738</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>382244</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" s="21" t="n"/>
-      <c r="I11" s="14" t="inlineStr">
+      <c r="G11" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="H11" s="23" t="n"/>
+      <c r="I11" s="15" t="inlineStr">
         <is>
           <t>20x25x2</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="K11" s="21" t="n">
+      <c r="K11" s="23" t="n">
         <v>4.83</v>
       </c>
-      <c r="L11" s="21">
+      <c r="L11" s="23">
         <f>J11*K11</f>
         <v/>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
         <is>
           <t>Delivered 2026-10-09</t>
         </is>
@@ -1897,7 +2008,7 @@
       <c r="N11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
@@ -1930,7 +2041,7 @@
       <c r="G12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H12" s="19" t="n"/>
+      <c r="H12" s="22" t="n"/>
       <c r="I12" s="11" t="inlineStr">
         <is>
           <t>20x20x4</t>
@@ -1939,10 +2050,10 @@
       <c r="J12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K12" s="22" t="n">
         <v>7.46</v>
       </c>
-      <c r="L12" s="19">
+      <c r="L12" s="22">
         <f>J12*K12</f>
         <v/>
       </c>
@@ -1951,59 +2062,59 @@
           <t>Delivered 2026-10-09</t>
         </is>
       </c>
-      <c r="N12" s="12" t="n"/>
+      <c r="N12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Angel Leon</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Tex Air Austin</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>770738</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>382244</t>
         </is>
       </c>
-      <c r="G13" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="H13" s="21" t="n"/>
-      <c r="I13" s="14" t="inlineStr">
+      <c r="G13" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" s="23" t="n"/>
+      <c r="I13" s="15" t="inlineStr">
         <is>
           <t>20x20x2</t>
         </is>
       </c>
-      <c r="J13" s="14" t="n">
+      <c r="J13" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="K13" s="21" t="n">
+      <c r="K13" s="23" t="n">
         <v>4.67</v>
       </c>
-      <c r="L13" s="21">
+      <c r="L13" s="23">
         <f>J13*K13</f>
         <v/>
       </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="M13" s="16" t="inlineStr">
         <is>
           <t>Delivered 2026-10-09</t>
         </is>
@@ -2011,383 +2122,383 @@
       <c r="N13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n"/>
+      <c r="A14" s="13" t="n"/>
       <c r="B14" s="12" t="n"/>
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="12" t="n"/>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
       <c r="G14" s="11" t="n"/>
-      <c r="H14" s="19" t="n"/>
+      <c r="H14" s="22" t="n"/>
       <c r="I14" s="11" t="n"/>
       <c r="J14" s="11" t="n"/>
-      <c r="K14" s="19" t="n"/>
-      <c r="L14" s="19">
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22">
         <f>IF(OR(J14="",K14=""),"",J14*K14)</f>
         <v/>
       </c>
       <c r="M14" s="12" t="n"/>
-      <c r="N14" s="12" t="n"/>
+      <c r="N14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="14" t="n"/>
-      <c r="J15" s="14" t="n"/>
-      <c r="K15" s="21" t="n"/>
-      <c r="L15" s="21">
+      <c r="A15" s="17" t="n"/>
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="23" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="23" t="n"/>
+      <c r="L15" s="23">
         <f>IF(OR(J15="",K15=""),"",J15*K15)</f>
         <v/>
       </c>
-      <c r="M15" s="7" t="n"/>
+      <c r="M15" s="16" t="n"/>
       <c r="N15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n"/>
+      <c r="A16" s="13" t="n"/>
       <c r="B16" s="12" t="n"/>
       <c r="C16" s="11" t="n"/>
       <c r="D16" s="12" t="n"/>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>
       <c r="G16" s="11" t="n"/>
-      <c r="H16" s="19" t="n"/>
+      <c r="H16" s="22" t="n"/>
       <c r="I16" s="11" t="n"/>
       <c r="J16" s="11" t="n"/>
-      <c r="K16" s="19" t="n"/>
-      <c r="L16" s="19">
+      <c r="K16" s="22" t="n"/>
+      <c r="L16" s="22">
         <f>IF(OR(J16="",K16=""),"",J16*K16)</f>
         <v/>
       </c>
       <c r="M16" s="12" t="n"/>
-      <c r="N16" s="12" t="n"/>
+      <c r="N16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="21" t="n"/>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="21" t="n"/>
-      <c r="L17" s="21">
+      <c r="A17" s="17" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="23" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="23" t="n"/>
+      <c r="L17" s="23">
         <f>IF(OR(J17="",K17=""),"",J17*K17)</f>
         <v/>
       </c>
-      <c r="M17" s="7" t="n"/>
+      <c r="M17" s="16" t="n"/>
       <c r="N17" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="n"/>
+      <c r="A18" s="13" t="n"/>
       <c r="B18" s="12" t="n"/>
       <c r="C18" s="11" t="n"/>
       <c r="D18" s="12" t="n"/>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
-      <c r="H18" s="19" t="n"/>
+      <c r="H18" s="22" t="n"/>
       <c r="I18" s="11" t="n"/>
       <c r="J18" s="11" t="n"/>
-      <c r="K18" s="19" t="n"/>
-      <c r="L18" s="19">
+      <c r="K18" s="22" t="n"/>
+      <c r="L18" s="22">
         <f>IF(OR(J18="",K18=""),"",J18*K18)</f>
         <v/>
       </c>
       <c r="M18" s="12" t="n"/>
-      <c r="N18" s="12" t="n"/>
+      <c r="N18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="21" t="n"/>
-      <c r="I19" s="14" t="n"/>
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="21" t="n"/>
-      <c r="L19" s="21">
+      <c r="A19" s="17" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="23" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="23" t="n"/>
+      <c r="L19" s="23">
         <f>IF(OR(J19="",K19=""),"",J19*K19)</f>
         <v/>
       </c>
-      <c r="M19" s="7" t="n"/>
+      <c r="M19" s="16" t="n"/>
       <c r="N19" s="7" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n"/>
+      <c r="A20" s="13" t="n"/>
       <c r="B20" s="12" t="n"/>
       <c r="C20" s="11" t="n"/>
       <c r="D20" s="12" t="n"/>
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
-      <c r="H20" s="19" t="n"/>
+      <c r="H20" s="22" t="n"/>
       <c r="I20" s="11" t="n"/>
       <c r="J20" s="11" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19">
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="22">
         <f>IF(OR(J20="",K20=""),"",J20*K20)</f>
         <v/>
       </c>
       <c r="M20" s="12" t="n"/>
-      <c r="N20" s="12" t="n"/>
+      <c r="N20" s="14" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="21" t="n"/>
-      <c r="I21" s="14" t="n"/>
-      <c r="J21" s="14" t="n"/>
-      <c r="K21" s="21" t="n"/>
-      <c r="L21" s="21">
+      <c r="A21" s="17" t="n"/>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="23" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="23" t="n"/>
+      <c r="L21" s="23">
         <f>IF(OR(J21="",K21=""),"",J21*K21)</f>
         <v/>
       </c>
-      <c r="M21" s="7" t="n"/>
+      <c r="M21" s="16" t="n"/>
       <c r="N21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="n"/>
+      <c r="A22" s="13" t="n"/>
       <c r="B22" s="12" t="n"/>
       <c r="C22" s="11" t="n"/>
       <c r="D22" s="12" t="n"/>
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
-      <c r="H22" s="19" t="n"/>
+      <c r="H22" s="22" t="n"/>
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19">
+      <c r="K22" s="22" t="n"/>
+      <c r="L22" s="22">
         <f>IF(OR(J22="",K22=""),"",J22*K22)</f>
         <v/>
       </c>
       <c r="M22" s="12" t="n"/>
-      <c r="N22" s="12" t="n"/>
+      <c r="N22" s="14" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="21" t="n"/>
-      <c r="I23" s="14" t="n"/>
-      <c r="J23" s="14" t="n"/>
-      <c r="K23" s="21" t="n"/>
-      <c r="L23" s="21">
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="23" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="23" t="n"/>
+      <c r="L23" s="23">
         <f>IF(OR(J23="",K23=""),"",J23*K23)</f>
         <v/>
       </c>
-      <c r="M23" s="7" t="n"/>
+      <c r="M23" s="16" t="n"/>
       <c r="N23" s="7" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="n"/>
+      <c r="A24" s="13" t="n"/>
       <c r="B24" s="12" t="n"/>
       <c r="C24" s="11" t="n"/>
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
-      <c r="H24" s="19" t="n"/>
+      <c r="H24" s="22" t="n"/>
       <c r="I24" s="11" t="n"/>
       <c r="J24" s="11" t="n"/>
-      <c r="K24" s="19" t="n"/>
-      <c r="L24" s="19">
+      <c r="K24" s="22" t="n"/>
+      <c r="L24" s="22">
         <f>IF(OR(J24="",K24=""),"",J24*K24)</f>
         <v/>
       </c>
       <c r="M24" s="12" t="n"/>
-      <c r="N24" s="12" t="n"/>
+      <c r="N24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="21" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
-      <c r="K25" s="21" t="n"/>
-      <c r="L25" s="21">
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="23" t="n"/>
+      <c r="I25" s="15" t="n"/>
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="23" t="n"/>
+      <c r="L25" s="23">
         <f>IF(OR(J25="",K25=""),"",J25*K25)</f>
         <v/>
       </c>
-      <c r="M25" s="7" t="n"/>
+      <c r="M25" s="16" t="n"/>
       <c r="N25" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="n"/>
+      <c r="A26" s="13" t="n"/>
       <c r="B26" s="12" t="n"/>
       <c r="C26" s="11" t="n"/>
       <c r="D26" s="12" t="n"/>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
-      <c r="H26" s="19" t="n"/>
+      <c r="H26" s="22" t="n"/>
       <c r="I26" s="11" t="n"/>
       <c r="J26" s="11" t="n"/>
-      <c r="K26" s="19" t="n"/>
-      <c r="L26" s="19">
+      <c r="K26" s="22" t="n"/>
+      <c r="L26" s="22">
         <f>IF(OR(J26="",K26=""),"",J26*K26)</f>
         <v/>
       </c>
       <c r="M26" s="12" t="n"/>
-      <c r="N26" s="12" t="n"/>
+      <c r="N26" s="14" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="n"/>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="14" t="n"/>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="21" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="14" t="n"/>
-      <c r="K27" s="21" t="n"/>
-      <c r="L27" s="21">
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="23" t="n"/>
+      <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="23" t="n"/>
+      <c r="L27" s="23">
         <f>IF(OR(J27="",K27=""),"",J27*K27)</f>
         <v/>
       </c>
-      <c r="M27" s="7" t="n"/>
+      <c r="M27" s="16" t="n"/>
       <c r="N27" s="7" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="n"/>
+      <c r="A28" s="13" t="n"/>
       <c r="B28" s="12" t="n"/>
       <c r="C28" s="11" t="n"/>
       <c r="D28" s="12" t="n"/>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
       <c r="G28" s="11" t="n"/>
-      <c r="H28" s="19" t="n"/>
+      <c r="H28" s="22" t="n"/>
       <c r="I28" s="11" t="n"/>
       <c r="J28" s="11" t="n"/>
-      <c r="K28" s="19" t="n"/>
-      <c r="L28" s="19">
+      <c r="K28" s="22" t="n"/>
+      <c r="L28" s="22">
         <f>IF(OR(J28="",K28=""),"",J28*K28)</f>
         <v/>
       </c>
       <c r="M28" s="12" t="n"/>
-      <c r="N28" s="12" t="n"/>
+      <c r="N28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="20" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="21" t="n"/>
-      <c r="I29" s="14" t="n"/>
-      <c r="J29" s="14" t="n"/>
-      <c r="K29" s="21" t="n"/>
-      <c r="L29" s="21">
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="23" t="n"/>
+      <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="23" t="n"/>
+      <c r="L29" s="23">
         <f>IF(OR(J29="",K29=""),"",J29*K29)</f>
         <v/>
       </c>
-      <c r="M29" s="7" t="n"/>
+      <c r="M29" s="16" t="n"/>
       <c r="N29" s="7" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="n"/>
+      <c r="A30" s="13" t="n"/>
       <c r="B30" s="12" t="n"/>
       <c r="C30" s="11" t="n"/>
       <c r="D30" s="12" t="n"/>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
-      <c r="H30" s="19" t="n"/>
+      <c r="H30" s="22" t="n"/>
       <c r="I30" s="11" t="n"/>
       <c r="J30" s="11" t="n"/>
-      <c r="K30" s="19" t="n"/>
-      <c r="L30" s="19">
+      <c r="K30" s="22" t="n"/>
+      <c r="L30" s="22">
         <f>IF(OR(J30="",K30=""),"",J30*K30)</f>
         <v/>
       </c>
       <c r="M30" s="12" t="n"/>
-      <c r="N30" s="12" t="n"/>
+      <c r="N30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="n"/>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="21" t="n"/>
-      <c r="I31" s="14" t="n"/>
-      <c r="J31" s="14" t="n"/>
-      <c r="K31" s="21" t="n"/>
-      <c r="L31" s="21">
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="23" t="n"/>
+      <c r="I31" s="15" t="n"/>
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="23" t="n"/>
+      <c r="L31" s="23">
         <f>IF(OR(J31="",K31=""),"",J31*K31)</f>
         <v/>
       </c>
-      <c r="M31" s="7" t="n"/>
+      <c r="M31" s="16" t="n"/>
       <c r="N31" s="7" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="n"/>
+      <c r="A32" s="13" t="n"/>
       <c r="B32" s="12" t="n"/>
       <c r="C32" s="11" t="n"/>
       <c r="D32" s="12" t="n"/>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
       <c r="G32" s="11" t="n"/>
-      <c r="H32" s="19" t="n"/>
+      <c r="H32" s="22" t="n"/>
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="11" t="n"/>
-      <c r="K32" s="19" t="n"/>
-      <c r="L32" s="19">
+      <c r="K32" s="22" t="n"/>
+      <c r="L32" s="22">
         <f>IF(OR(J32="",K32=""),"",J32*K32)</f>
         <v/>
       </c>
       <c r="M32" s="12" t="n"/>
-      <c r="N32" s="12" t="n"/>
+      <c r="N32" s="14" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="20" t="n"/>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="21" t="n"/>
-      <c r="I33" s="14" t="n"/>
-      <c r="J33" s="14" t="n"/>
-      <c r="K33" s="21" t="n"/>
-      <c r="L33" s="21">
+      <c r="A33" s="17" t="n"/>
+      <c r="B33" s="16" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="23" t="n"/>
+      <c r="I33" s="15" t="n"/>
+      <c r="J33" s="15" t="n"/>
+      <c r="K33" s="23" t="n"/>
+      <c r="L33" s="23">
         <f>IF(OR(J33="",K33=""),"",J33*K33)</f>
         <v/>
       </c>
-      <c r="M33" s="7" t="n"/>
+      <c r="M33" s="16" t="n"/>
       <c r="N33" s="7" t="n"/>
     </row>
   </sheetData>

</xml_diff>